<commit_message>
feat(generator): add enterprise reference data configuration sheet
</commit_message>
<xml_diff>
--- a/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
+++ b/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
@@ -23,8 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +45,12 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -57,7 +65,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,16 +73,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -149,6 +182,34 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ChangeRegisterTable" displayName="ChangeRegisterTable" ref="A3:S4" headerRowCount="1">
+  <autoFilter ref="A3:S4"/>
+  <tableColumns count="19">
+    <tableColumn id="1" name="Change ID"/>
+    <tableColumn id="2" name="Change Title"/>
+    <tableColumn id="3" name="Change Category"/>
+    <tableColumn id="4" name="Change Type"/>
+    <tableColumn id="5" name="Status"/>
+    <tableColumn id="6" name="Risk Level"/>
+    <tableColumn id="7" name="Priority"/>
+    <tableColumn id="8" name="Linked CI ID"/>
+    <tableColumn id="9" name="Asset ID"/>
+    <tableColumn id="10" name="Requested By"/>
+    <tableColumn id="11" name="Assigned Engineer"/>
+    <tableColumn id="12" name="CAB Approval"/>
+    <tableColumn id="13" name="Planned Start"/>
+    <tableColumn id="14" name="Planned End"/>
+    <tableColumn id="15" name="Actual Start"/>
+    <tableColumn id="16" name="Actual End"/>
+    <tableColumn id="17" name="Rollback Plan"/>
+    <tableColumn id="18" name="Validation Status"/>
+    <tableColumn id="19" name="Comments"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -607,10 +668,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROJECT ORION — ENTERPRISE CHANGE REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Governed tracking of infrastructure, security, application, and operational changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Change ID</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Change Title</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Change Category</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Change Type</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Risk Level</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Linked CI ID</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Asset ID</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Requested By</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Assigned Engineer</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>CAB Approval</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Planned Start</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Planned End</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Actual Start</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>Actual End</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>Rollback Plan</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
+      <c r="Q4" s="5" t="n"/>
+      <c r="R4" s="5" t="n"/>
+      <c r="S4" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -659,9 +881,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Change Type</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Risk Level</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>CAB Approval</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(generator): implement enterprise data validation dropdowns
</commit_message>
<xml_diff>
--- a/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
+++ b/docs/engineering/change-management/PO-CHANGE-REGISTER_v1.0.xlsx
@@ -12,9 +12,9 @@
     <sheet name="02_Change_History" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03_CAB_Meetings" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="04_Implementation_Checklist" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05_Reference_Data" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06_Revision_History" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07_Dashboard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="07_Dashboard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="05_Reference_Data" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="06_Revision_History" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -829,6 +829,32 @@
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A1:S1"/>
   </mergeCells>
+  <dataValidations count="8">
+    <dataValidation sqref="C4:C503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$M$2:$M$9</formula1>
+    </dataValidation>
+    <dataValidation sqref="D4:D503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$A$2:$A$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$C$2:$C$6</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$G$2:$G$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="G4:G503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$E$2:$E$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="L4:L503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$I$2:$I$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q4:Q503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$O$2:$O$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="R4:R503" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Selection" error="Select a value from the approved dropdown list." promptTitle="Controlled Value" prompt="Choose an approved Project Orion value." type="list">
+      <formula1>='05_Reference_Data'!$K$2:$K$5</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -881,175 +907,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Change Type</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Risk Level</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>CAB Approval</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>Validation Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Emergency</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Cancelled</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1060,9 +920,243 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Change Type</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Risk Level</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>CAB Approval</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Validation Status</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>Change Category</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t>Rollback Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>